<commit_message>
fix: update template import hapus kolom NIPD
</commit_message>
<xml_diff>
--- a/static/template-import-santri.xlsx
+++ b/static/template-import-santri.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Aldi Nitip\Hady Nitip\Project\buku-induk\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SERVER\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCD1C112-C551-47B5-B37A-821784601D80}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31968A3D-3A73-4FCE-B779-C8F03524DD3C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
     <author>SERVER</author>
   </authors>
   <commentList>
-    <comment ref="Z1" authorId="0" shapeId="0" xr:uid="{D229EC09-8403-48DD-BC88-E86B30C2CCBF}">
+    <comment ref="X1" authorId="0" shapeId="0" xr:uid="{D229EC09-8403-48DD-BC88-E86B30C2CCBF}">
       <text>
         <r>
           <rPr>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="54">
   <si>
     <t>Nama lengkap *</t>
   </si>
@@ -69,9 +69,6 @@
     <t>NIS</t>
   </si>
   <si>
-    <t>NIPD</t>
-  </si>
-  <si>
     <t>Nama panggilan</t>
   </si>
   <si>
@@ -85,9 +82,6 @@
   </si>
   <si>
     <t>Agama</t>
-  </si>
-  <si>
-    <t>Kewarganegaraan</t>
   </si>
   <si>
     <t>Tempat tinggal</t>
@@ -639,48 +633,46 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AM1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AK1"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="4.875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="3.75" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="3.625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="11.625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="6.5" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="6.875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="3.875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.25" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="10.125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="7.875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="6.375" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="13.875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="3.875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.25" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="6.375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="13.375" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="11.375" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="13.375" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="10.75" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="13.625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="13.125" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="10.375" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="9.75" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="13.75" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="12.375" bestFit="1" customWidth="1"/>
-    <col min="37" max="38" width="10.875" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="10.375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="10.75" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="13.625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="13.125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="10.375" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="9.75" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="13.75" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="10.875" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="10.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:37" s="1" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -791,18 +783,12 @@
       </c>
       <c r="AK1" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="AL1" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM1" s="2" t="s">
-        <v>38</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:AM1" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:D1 E1:I1 J1:AK1" numberStoredAsText="1"/>
   </ignoredErrors>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
@@ -811,84 +797,84 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="B12" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="C12" t="s">
         <v>49</v>
       </c>
-      <c r="B12" t="s">
+      <c r="D12" t="s">
         <v>50</v>
       </c>
-      <c r="C12" t="s">
+      <c r="E12" t="s">
         <v>51</v>
       </c>
-      <c r="D12" t="s">
+      <c r="F12" t="s">
         <v>52</v>
       </c>
-      <c r="E12" t="s">
+      <c r="G12" t="s">
         <v>53</v>
-      </c>
-      <c r="F12" t="s">
-        <v>54</v>
-      </c>
-      <c r="G12" t="s">
-        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: kolom NIS di sheet data opsional sebagai kunci verifikasi baris antar-sheet
</commit_message>
<xml_diff>
--- a/static/template-import-santri.xlsx
+++ b/static/template-import-santri.xlsx
@@ -439,104 +439,107 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AC1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>NIS</v>
+      </c>
+      <c r="B1" t="str">
         <v>NIK</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
         <v>Nama panggilan</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Agama</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Tempat tinggal</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Transportasi</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Anak ke</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>No. HP</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>RT</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>RW</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Desa/kelurahan</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Kecamatan</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Kabupaten</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>No. akta</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>No. KK</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>Bantuan (KIP/PIP/KPS/PKH)</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>Status keluarga</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>Status santri</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>Tanggal masuk</v>
       </c>
-      <c r="S1" t="str">
+      <c r="T1" t="str">
         <v>Asal sekolah</v>
       </c>
-      <c r="T1" t="str">
+      <c r="U1" t="str">
         <v>Jalur masuk</v>
       </c>
-      <c r="U1" t="str">
+      <c r="V1" t="str">
         <v>Kamar (nomor)</v>
       </c>
-      <c r="V1" t="str">
+      <c r="W1" t="str">
         <v>Kelas (mis. 7A)</v>
       </c>
-      <c r="W1" t="str">
+      <c r="X1" t="str">
         <v>Nama wali</v>
       </c>
-      <c r="X1" t="str">
+      <c r="Y1" t="str">
         <v>Pekerjaan ayah</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="Z1" t="str">
         <v>Pekerjaan ibu</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AA1" t="str">
         <v>Penghasilan</v>
       </c>
-      <c r="AA1" t="str">
+      <c r="AB1" t="str">
         <v>Alamat wali</v>
       </c>
-      <c r="AB1" t="str">
+      <c r="AC1" t="str">
         <v>No. HP wali</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AC1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -560,110 +563,115 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>3. Kolom wajib (Nama, NIS, NISN, Jenis Kelamin, Tempat Lahir, Tanggal Lahir, Alamat, Nama Ayah, Nama Ibu) sebaiknya terisi semua; sisanya opsional.</v>
+        <v>3. Kolom NIS ada di KEDUA sheet sebagai kunci pencocokan — isinya harus sama. Kalau berbeda, baris tersebut ditolak saat import.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>4. Jenis kelamin: L atau P</v>
+        <v>4. Kolom wajib (Nama, NIS, NISN, Jenis Kelamin, Tempat Lahir, Tanggal Lahir, Alamat, Nama Ayah, Nama Ibu) sebaiknya terisi semua; sisanya opsional.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>5. RT/RW otomatis jadi 3 digit (contoh: 9 atau 09 tersimpan sebagai 009).</v>
+        <v>5. Jenis kelamin: L atau P</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>6. Tanggal lahir bebas formatnya: 10/11/2026, 10-11-2026, atau 10 November 2026 — otomatis dirapikan sistem.</v>
+        <v>6. RT/RW otomatis jadi 3 digit (contoh: 9 atau 09 tersimpan sebagai 009).</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>7. Status santri: aktif, khusus, mutasi_keluar, lulus, wafat, drop_out</v>
+        <v>7. Tanggal lahir bebas formatnya: 10/11/2026, 10-11-2026, atau 10 November 2026 — otomatis dirapikan sistem.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>8. Status keluarga: yatim, yatim_piatu, dhuafa, umum</v>
+        <v>8. Status santri: aktif, khusus, mutasi_keluar, lulus, wafat, drop_out</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>9. Kamar: nomor kamar (contoh: 3). Kelas: tingkat+rombel (contoh: 7A).</v>
+        <v>9. Status keluarga: yatim, yatim_piatu, dhuafa, umum</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v/>
+        <v>10. Kamar: nomor kamar (contoh: 3). Kelas: tingkat+rombel (contoh: 7A).</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Contoh baris 2 sheet "data wajib":</v>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Nama lengkap</v>
-      </c>
-      <c r="B14" t="str">
-        <v>NIS</v>
-      </c>
-      <c r="C14" t="str">
-        <v>NISN</v>
-      </c>
-      <c r="D14" t="str">
-        <v>Jenis kelamin (L/P)</v>
-      </c>
-      <c r="E14" t="str">
-        <v>Tempat lahir</v>
-      </c>
-      <c r="F14" t="str">
-        <v>Tanggal lahir</v>
-      </c>
-      <c r="G14" t="str">
-        <v>Alamat</v>
-      </c>
-      <c r="H14" t="str">
-        <v>Nama ayah</v>
-      </c>
-      <c r="I14" t="str">
-        <v>Nama ibu</v>
+        <v>Contoh baris 2 sheet "data wajib":</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
+        <v>Nama lengkap</v>
+      </c>
+      <c r="B15" t="str">
+        <v>NIS</v>
+      </c>
+      <c r="C15" t="str">
+        <v>NISN</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Jenis kelamin (L/P)</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Tempat lahir</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Tanggal lahir</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Alamat</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Nama ayah</v>
+      </c>
+      <c r="I15" t="str">
+        <v>Nama ibu</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
         <v>Ahmad Fauzi</v>
       </c>
-      <c r="B15" t="str">
+      <c r="B16" t="str">
         <v>2410001</v>
       </c>
-      <c r="C15" t="str">
+      <c r="C16" t="str">
         <v>0012345678</v>
       </c>
-      <c r="D15" t="str">
+      <c r="D16" t="str">
         <v>L</v>
       </c>
-      <c r="E15" t="str">
+      <c r="E16" t="str">
         <v>Yogyakarta</v>
       </c>
-      <c r="F15" t="str">
+      <c r="F16" t="str">
         <v>10 November 2010</v>
       </c>
-      <c r="G15" t="str">
+      <c r="G16" t="str">
         <v>Jl. Kaliurang No. 9 RT 009 RW 012</v>
       </c>
-      <c r="H15" t="str">
+      <c r="H16" t="str">
         <v>Haji Salim</v>
       </c>
-      <c r="I15" t="str">
+      <c r="I16" t="str">
         <v>Siti Aminah</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: import fleksibel — sheet opsional boleh kosong/hanya NIS, cocokkan by NIS bukan posisi baris
</commit_message>
<xml_diff>
--- a/static/template-import-santri.xlsx
+++ b/static/template-import-santri.xlsx
@@ -539,7 +539,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -558,120 +558,125 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2. Baris di kedua sheet harus sejajar: baris 2 "data wajib" dan baris 2 "data opsional" adalah santri yang sama.</v>
+        <v>2. Sheet "data wajib" WAJIB diisi (9 kolom). Sheet "data opsional" boleh kosong total, hanya isi NIS, atau penuh.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>3. Kolom NIS ada di KEDUA sheet sebagai kunci pencocokan — isinya harus sama. Kalau berbeda, baris tersebut ditolak saat import.</v>
+        <v>3. Jika "data opsional" diisi NIS-nya, sistem otomatis cocokkan dengan NIS di "data wajib" (tidak perlu urut sama).</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>4. Kolom wajib (Nama, NIS, NISN, Jenis Kelamin, Tempat Lahir, Tanggal Lahir, Alamat, Nama Ayah, Nama Ibu) sebaiknya terisi semua; sisanya opsional.</v>
+        <v>4. Kolom NIS ada di KEDUA sheet sebagai kunci pencocokan — isinya harus sama bila keduanya diisi.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>5. Jenis kelamin: L atau P</v>
+        <v>5. Kolom wajib (Nama, NIS, NISN, Jenis Kelamin, Tempat Lahir, Tanggal Lahir, Alamat, Nama Ayah, Nama Ibu) sebaiknya terisi semua; sisanya opsional.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>6. RT/RW otomatis jadi 3 digit (contoh: 9 atau 09 tersimpan sebagai 009).</v>
+        <v>6. Jenis kelamin: L atau P</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>7. Tanggal lahir bebas formatnya: 10/11/2026, 10-11-2026, atau 10 November 2026 — otomatis dirapikan sistem.</v>
+        <v>7. RT/RW otomatis jadi 3 digit (contoh: 9 atau 09 tersimpan sebagai 009).</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>8. Status santri: aktif, khusus, mutasi_keluar, lulus, wafat, drop_out</v>
+        <v>8. Tanggal lahir bebas formatnya: 10/11/2026, 10-11-2026, atau 10 November 2026 — otomatis dirapikan sistem.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>9. Status keluarga: yatim, yatim_piatu, dhuafa, umum</v>
+        <v>9. Status santri: aktif, khusus, mutasi_keluar, lulus, wafat, drop_out</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>10. Kamar: nomor kamar (contoh: 3). Kelas: tingkat+rombel (contoh: 7A).</v>
+        <v>10. Status keluarga: yatim, yatim_piatu, dhuafa, umum</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v/>
+        <v>11. Kamar: nomor kamar (contoh: 3). Kelas: tingkat+rombel (contoh: 7A).</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Contoh baris 2 sheet "data wajib":</v>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Nama lengkap</v>
-      </c>
-      <c r="B15" t="str">
-        <v>NIS</v>
-      </c>
-      <c r="C15" t="str">
-        <v>NISN</v>
-      </c>
-      <c r="D15" t="str">
-        <v>Jenis kelamin (L/P)</v>
-      </c>
-      <c r="E15" t="str">
-        <v>Tempat lahir</v>
-      </c>
-      <c r="F15" t="str">
-        <v>Tanggal lahir</v>
-      </c>
-      <c r="G15" t="str">
-        <v>Alamat</v>
-      </c>
-      <c r="H15" t="str">
-        <v>Nama ayah</v>
-      </c>
-      <c r="I15" t="str">
-        <v>Nama ibu</v>
+        <v>Contoh baris 2 sheet "data wajib":</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
+        <v>Nama lengkap</v>
+      </c>
+      <c r="B16" t="str">
+        <v>NIS</v>
+      </c>
+      <c r="C16" t="str">
+        <v>NISN</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Jenis kelamin (L/P)</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Tempat lahir</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Tanggal lahir</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Alamat</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Nama ayah</v>
+      </c>
+      <c r="I16" t="str">
+        <v>Nama ibu</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
         <v>Ahmad Fauzi</v>
       </c>
-      <c r="B16" t="str">
+      <c r="B17" t="str">
         <v>2410001</v>
       </c>
-      <c r="C16" t="str">
+      <c r="C17" t="str">
         <v>0012345678</v>
       </c>
-      <c r="D16" t="str">
+      <c r="D17" t="str">
         <v>L</v>
       </c>
-      <c r="E16" t="str">
+      <c r="E17" t="str">
         <v>Yogyakarta</v>
       </c>
-      <c r="F16" t="str">
+      <c r="F17" t="str">
         <v>10 November 2010</v>
       </c>
-      <c r="G16" t="str">
+      <c r="G17" t="str">
         <v>Jl. Kaliurang No. 9 RT 009 RW 012</v>
       </c>
-      <c r="H16" t="str">
+      <c r="H17" t="str">
         <v>Haji Salim</v>
       </c>
-      <c r="I16" t="str">
+      <c r="I17" t="str">
         <v>Siti Aminah</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>